<commit_message>
feat(sprint-4): enhance UX/UI with Plotly charts, dynamic progress bar, ETA, and direct Excel download
</commit_message>
<xml_diff>
--- a/output/LinkedIn_BA_France_Report.xlsx
+++ b/output/LinkedIn_BA_France_Report.xlsx
@@ -456,13 +456,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
@@ -535,32 +535,32 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Software Engineer (Azure)</t>
+          <t>Apprenti, Business &amp; Data Analyst (F/H)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Norrin</t>
+          <t>Del Monte Corporation</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>17 hours ago</t>
+          <t>2 hours ago</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/jobs/view/software-engineer-azure-at-norrin-4368032456</t>
+          <t>https://fr.linkedin.com/jobs/view/apprenti-business-data-analyst-f-h-at-del-monte-corporation-4456874561</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>SAP, SAFe, DevOps, Compétences en communication, Résolution de problèmes, Anglais</t>
+          <t>Power BI, Excel, MS Visio</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\1_Norrin_Software_Engineer_(Azure).png</t>
+          <t>output\screenshots\1_Del_Monte_Corporation_Apprenti,_Business_&amp;_Data_Analyst_(F_H).png</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -578,32 +578,32 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Junior Software Engineer (C/C++, Linux)</t>
+          <t>Alternance 12 à 24 mois - Chargé projet digital (H/F)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Endava</t>
+          <t>OCP Répartition</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>19 hours ago</t>
+          <t>21 hours ago</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/jobs/view/junior-software-engineer-c-c%2B%2B-linux-at-endava-4453921223</t>
+          <t>https://fr.linkedin.com/jobs/view/alternance-12-%C3%A0-24-mois-charg%C3%A9-projet-digital-h-f-at-ocp-r%C3%A9partition-4420446757</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Agile, SAFe, Compétences en communication, Anglais</t>
+          <t>Power BI, Excel, Python, R</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\2_Endava_Junior_Software_Engineer_(C_C++,_Linux).png</t>
+          <t>output\screenshots\2_OCP_Répartition_Alternance_12_à_24_mois_-_Chargé_projet_digital_(H_F).png</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -621,32 +621,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Tech Lead - HCM</t>
+          <t>Business Analyst @eXalt Ouest</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>XCapital Technology</t>
+          <t>eXalt</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>18 hours ago</t>
+          <t>23 hours ago</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/jobs/view/tech-lead-hcm-at-xcapital-technology-4453914335</t>
+          <t>https://fr.linkedin.com/jobs/view/business-analyst-%40exalt-ouest-at-exalt-4420550474</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Python, Recueil des besoins</t>
+          <t>Excel, Gestion des parties prenantes, Recueil des besoins, Gestion de projet, Anglais</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\3_XCapital_Technology_Tech_Lead_-_HCM.png</t>
+          <t>output\screenshots\3_eXalt_Business_Analyst_@eXalt_Ouest.png</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -664,32 +664,32 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Senior 3D Web Engineer</t>
+          <t>Alternant Data Gouvernance Officer (F/H)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Symbotic</t>
+          <t>BMW Group</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>15 hours ago</t>
+          <t>44 minutes ago</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/jobs/view/senior-3d-web-engineer-at-symbotic-4416906345</t>
+          <t>https://fr.linkedin.com/jobs/view/alternant-data-gouvernance-officer-f-h-at-bmw-group-4456886776</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Excel, Gestion des parties prenantes, Recueil des besoins, Compétences en communication, Anglais</t>
+          <t>SQL, Python, Tableau, Recueil des besoins, Compétences en communication</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\4_Symbotic_Senior_3D_Web_Engineer.png</t>
+          <t>output\screenshots\4_BMW_Group_Alternant_Data_Gouvernance_Officer_(F_H).png</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -707,32 +707,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Senior Mobile Developer (iOS/Android)</t>
+          <t>Business Analyst F/H</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>VinSmart Future</t>
+          <t>CGI</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>21 hours ago</t>
+          <t>23 hours ago</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/jobs/view/senior-mobile-developer-ios-android-at-vinsmart-future-4450889252</t>
+          <t>https://fr.linkedin.com/jobs/view/business-analyst-f-h-at-cgi-4390659826</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Excel, Recueil des besoins</t>
+          <t>Excel, Recueil des besoins, Compétences en communication</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\5_VinSmart_Future_Senior_Mobile_Developer_(iOS_Android).png</t>
+          <t>output\screenshots\5_CGI_Business_Analyst_F_H.png</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -750,32 +750,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Senior Software Development Engineer in Test - SDET</t>
+          <t>Alternance – Data Analyst (H/F)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>NVIDIA</t>
+          <t>Alltricks</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>15 hours ago</t>
+          <t>1 hour ago</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>https://vn.linkedin.com/jobs/view/senior-software-development-engineer-in-test-sdet-at-nvidia-4435293111</t>
+          <t>https://fr.linkedin.com/jobs/view/alternance-%E2%80%93-data-analyst-h-f-at-alltricks-4456876625</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Excel, Python, MS Visio, Recueil des besoins, Analyse de données, Anglais</t>
+          <t>Excel, Tableau, Salesforce, Recueil des besoins</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\6_NVIDIA_Senior_Software_Development_Engineer_in_Test_-_SDET.png</t>
+          <t>output\screenshots\6_Alltricks_Alternance_–_Data_Analyst_(H_F).png</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -787,9 +787,353 @@
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr"/>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Business Analyst (H/F)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Davidson consulting</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1 hour ago</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/business-analyst-h-f-at-davidson-consulting-4342654913</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SQL, Jira, Confluence, Agile, Scrum, Gestion des parties prenantes, Recueil des besoins</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>output\screenshots\7_Davidson_consulting_Business_Analyst_(H_F).png</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="3" t="inlineStr"/>
+      <c r="K8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Business Analyst Salesforce (H/F)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>YEVO</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>23 hours ago</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/business-analyst-salesforce-h-f-at-yevo-4456807402</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Excel, Jira, Tableau, UML, Salesforce, Confluence, Agile, Scrum, Gestion des parties prenantes, Recueil des besoins, Gestion de projet, Compétences en communication</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>output\screenshots\8_YEVO_Business_Analyst_Salesforce_(H_F).png</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="3" t="inlineStr"/>
+      <c r="K9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Business analyst</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Bending Spoons</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>19 hours ago</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/business-analyst-at-bending-spoons-4456804682</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Excel, Anglais</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>output\screenshots\9_Bending_Spoons_Business_analyst.png</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="3" t="inlineStr"/>
+      <c r="K10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Data Analyst</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>papernest</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>5 hours ago</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/data-analyst-at-papernest-4458178575</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>SQL, Tableau, Français, Anglais</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>output\screenshots\10_papernest_Data_Analyst.png</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="3" t="inlineStr"/>
+      <c r="K11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Business Analyst - Base de données</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>act digital EMEA - Alter Solutions</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>9 hours ago</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/business-analyst-base-de-donn%C3%A9es-at-act-digital-emea-alter-solutions-4455826741</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SQL, MS Visio, Agile, Gestion des parties prenantes, Recueil des besoins</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>output\screenshots\11_act_digital_EMEA_-_Alter_Solutions_Business_Analyst_-_Base_de_données.png</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="3" t="inlineStr"/>
+      <c r="K12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Business Analyst Fonctionnel - Toulouse- F/H</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Free-Work</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>4 hours ago</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/business-analyst-fonctionnel-toulouse-f-h-at-free-work-4455849523</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Excel, SAP, Agile, Scrum, Gestion des parties prenantes, Recueil des besoins, Gestion de projet</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>output\screenshots\12_Free-Work_Business_Analyst_Fonctionnel_-_Toulouse-_F_H.png</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="3" t="inlineStr"/>
+      <c r="K13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Business Analyst / Consultant E-Commerce (H/F)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>SQLI</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>21 hours ago</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/business-analyst-consultant-e-commerce-h-f-at-sqli-4390330065</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SQL, Recueil des besoins, Compétences en communication</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>output\screenshots\13_SQLI_Business_Analyst_Consultant_E-Commerce_(H_F).png</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="3" t="inlineStr"/>
+      <c r="K14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Business Analyste technique – Assurance non vie (F/H)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>BPCE Solutions informatiques</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>4 hours ago</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>https://fr.linkedin.com/jobs/view/business-analyste-technique-%E2%80%93-assurance-non-vie-f-h-at-bpce-solutions-informatiques-4428504183</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Jira, Confluence, MS Visio, Agile, DevOps, Recueil des besoins, Compétences en communication, Français, Anglais</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>output\screenshots\14_BPCE_Solutions_informatiques_Business_Analyste_technique_–_Assurance_non_vie_(F_H).png</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>À postuler</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="3" t="inlineStr"/>
+      <c r="K15" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Erreur" error="Saisie non valide" promptTitle="Statut Candidature" prompt="Veuillez choisir un statut dans la liste" type="list">
+    <dataValidation sqref="H2:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Erreur" error="Saisie non valide" promptTitle="Statut Candidature" prompt="Veuillez choisir un statut dans la liste" type="list">
       <formula1>"À postuler,Postulé,Entretien,Refusé,Offre reçue"</formula1>
     </dataValidation>
   </dataValidations>
@@ -806,6 +1150,22 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -817,7 +1177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -862,20 +1222,20 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Anglais</t>
+          <t>Recueil des besoins</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Langue</t>
+          <t>Compétence Professionnelle / Soft Skill</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>71.4%</t>
         </is>
       </c>
     </row>
@@ -887,20 +1247,20 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Recueil des besoins</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Compétence Professionnelle / Soft Skill</t>
+          <t>Outil Technique / Logiciel</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>66.7%</t>
+          <t>57.1%</t>
         </is>
       </c>
     </row>
@@ -912,7 +1272,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>SQL</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -921,11 +1281,11 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>35.7%</t>
         </is>
       </c>
     </row>
@@ -937,7 +1297,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Compétences en communication</t>
+          <t>Gestion des parties prenantes</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -946,11 +1306,11 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>35.7%</t>
         </is>
       </c>
     </row>
@@ -962,20 +1322,20 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>SAFe</t>
+          <t>Compétences en communication</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Méthodologie / Framework</t>
+          <t>Compétence Professionnelle / Soft Skill</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>35.7%</t>
         </is>
       </c>
     </row>
@@ -987,20 +1347,20 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>Agile</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Outil Technique / Logiciel</t>
+          <t>Méthodologie / Framework</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>35.7%</t>
         </is>
       </c>
     </row>
@@ -1012,20 +1372,20 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Résolution de problèmes</t>
+          <t>Tableau</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Compétence Professionnelle / Soft Skill</t>
+          <t>Outil Technique / Logiciel</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -1037,20 +1397,20 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>SAP</t>
+          <t>Anglais</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Outil Technique / Logiciel</t>
+          <t>Langue</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>28.6%</t>
         </is>
       </c>
     </row>
@@ -1062,20 +1422,20 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>DevOps</t>
+          <t>MS Visio</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Méthodologie / Framework</t>
+          <t>Outil Technique / Logiciel</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
@@ -1087,20 +1447,20 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Agile</t>
+          <t>Confluence</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Méthodologie / Framework</t>
+          <t>Outil Technique / Logiciel</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
@@ -1112,20 +1472,20 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Gestion des parties prenantes</t>
+          <t>Jira</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Compétence Professionnelle / Soft Skill</t>
+          <t>Outil Technique / Logiciel</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
@@ -1137,20 +1497,20 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>MS Visio</t>
+          <t>Scrum</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Outil Technique / Logiciel</t>
+          <t>Méthodologie / Framework</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>16.7%</t>
+          <t>21.4%</t>
         </is>
       </c>
     </row>
@@ -1162,7 +1522,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Analyse de données</t>
+          <t>Gestion de projet</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1171,11 +1531,211 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>21.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Top 14</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Français</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Langue</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Top 15</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Outil Technique / Logiciel</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Top 16</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Power BI</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Outil Technique / Logiciel</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Top 17</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Salesforce</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Outil Technique / Logiciel</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>14.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Top 18</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Outil Technique / Logiciel</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>16.7%</t>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>7.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Top 19</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>UML</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Outil Technique / Logiciel</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>7.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Top 20</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>SAP</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Outil Technique / Logiciel</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>7.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Top 21</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>DevOps</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Méthodologie / Framework</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>7.1%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(sprint-4): optimize scraper performance, fix chart formatting and add native job viewer
</commit_message>
<xml_diff>
--- a/output/LinkedIn_BA_France_Report.xlsx
+++ b/output/LinkedIn_BA_France_Report.xlsx
@@ -18,13 +18,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -51,13 +54,19 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
     <border>
       <left style="thin">
@@ -79,16 +88,16 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -456,13 +465,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="44" customWidth="1" min="5" max="5"/>
     <col width="44" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
@@ -535,32 +544,32 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Apprenti, Business &amp; Data Analyst (F/H)</t>
+          <t>Alternance - Business Process Owner Inventory</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Del Monte Corporation</t>
+          <t>CEVA SANTE ANIMALE</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>2 hours ago</t>
+          <t>5 hours ago</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/apprenti-business-data-analyst-f-h-at-del-monte-corporation-4456874561</t>
+          <t>https://fr.linkedin.com/jobs/view/alternance-business-process-owner-inventory-at-ceva-sante-animale-4422270589</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>Power BI, Excel, MS Visio</t>
+          <t>Power BI, Excel, MS Visio, Gestion du changement, Analyse de données, Français, Anglais</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\1_Del_Monte_Corporation_Apprenti,_Business_&amp;_Data_Analyst_(F_H).png</t>
+          <t>output\screenshots\1_CEVA_SANTE_ANIMALE_Alternance_-_Business_Process_Owner_Inventory.png</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -578,32 +587,32 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Alternance 12 à 24 mois - Chargé projet digital (H/F)</t>
+          <t>FBNL Stage - Business Analyst Junior - Data, Power BI &amp; AI H/F/X</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>OCP Répartition</t>
+          <t>The Estée Lauder Companies Inc.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>21 hours ago</t>
+          <t>5 hours ago</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/alternance-12-%C3%A0-24-mois-charg%C3%A9-projet-digital-h-f-at-ocp-r%C3%A9partition-4420446757</t>
+          <t>https://fr.linkedin.com/jobs/view/fbnl-stage-business-analyst-junior-data-power-bi-ai-h-f-x-at-the-est%C3%A9e-lauder-companies-inc-4461661452</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Power BI, Excel, Python, R</t>
+          <t>SQL, Power BI, Excel, Analyse de données, Anglais</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\2_OCP_Répartition_Alternance_12_à_24_mois_-_Chargé_projet_digital_(H_F).png</t>
+          <t>output\screenshots\2_The_Estée_Lauder_Companies_Inc._FBNL_Stage_-_Business_Analyst_Junior_-_Data,_Power_BI_&amp;_AI_H_F_X.png</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -621,32 +630,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Business Analyst @eXalt Ouest</t>
+          <t>Consultant Alternant IT &amp; Programmes de Transformation d'Entreprise F/H</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>eXalt</t>
+          <t>KPMG France</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>23 hours ago</t>
+          <t>4 hours ago</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/business-analyst-%40exalt-ouest-at-exalt-4420550474</t>
+          <t>https://fr.linkedin.com/jobs/view/consultant-alternant-it-programmes-de-transformation-d-entreprise-f-h-at-kpmg-france-4441439386</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Excel, Gestion des parties prenantes, Recueil des besoins, Gestion de projet, Anglais</t>
+          <t>Excel, Tableau, MS Visio, PowerPoint, Gestion de projet, Anglais</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\3_eXalt_Business_Analyst_@eXalt_Ouest.png</t>
+          <t>output\screenshots\3_KPMG_France_Consultant_Alternant_IT_&amp;_Programmes_de_Transformation_d'Entreprise_F_H.png</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -664,32 +673,32 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Alternant Data Gouvernance Officer (F/H)</t>
+          <t>Alternance Ingénieur d'Affaires F/H F/H</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>BMW Group</t>
+          <t>VINCI Energies</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>44 minutes ago</t>
+          <t>7 hours ago</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/alternant-data-gouvernance-officer-f-h-at-bmw-group-4456886776</t>
+          <t>https://fr.linkedin.com/jobs/view/alternance-ing%C3%A9nieur-d-affaires-f-h-f-h-at-vinci-energies-4463333910</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>SQL, Python, Tableau, Recueil des besoins, Compétences en communication</t>
+          <t>MS Visio, R, Gestion des parties prenantes, Recueil des besoins, Gestion de projet, Anglais</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\4_BMW_Group_Alternant_Data_Gouvernance_Officer_(F_H).png</t>
+          <t>output\screenshots\4_VINCI_Energies_Alternance_Ingénieur_d'Affaires_F_H_F_H.png</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -707,32 +716,32 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Business Analyst F/H</t>
+          <t>Appui en Référentiels SI et Architecture (H/F) - Alternance</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>CGI</t>
+          <t>Allianz France</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>23 hours ago</t>
+          <t>10 hours ago</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/business-analyst-f-h-at-cgi-4390659826</t>
+          <t>https://fr.linkedin.com/jobs/view/appui-en-r%C3%A9f%C3%A9rentiels-si-et-architecture-h-f-alternance-at-allianz-france-4443910062</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Excel, Recueil des besoins, Compétences en communication</t>
+          <t>Power BI, Tableau, SharePoint, Compétences en communication, Anglais</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\5_CGI_Business_Analyst_F_H.png</t>
+          <t>output\screenshots\5_Allianz_France_Appui_en_Référentiels_SI_et_Architecture_(H_F)_-_Alternance.png</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -750,32 +759,32 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Alternance – Data Analyst (H/F)</t>
+          <t>Stage Business Analyst F/H</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Alltricks</t>
+          <t>Galeries Lafayette</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>1 hour ago</t>
+          <t>5 hours ago</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>https://fr.linkedin.com/jobs/view/alternance-%E2%80%93-data-analyst-h-f-at-alltricks-4456876625</t>
+          <t>https://fr.linkedin.com/jobs/view/stage-business-analyst-f-h-at-galeries-lafayette-4463381202</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Excel, Tableau, Salesforce, Recueil des besoins</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>output\screenshots\6_Alltricks_Alternance_–_Data_Analyst_(H_F).png</t>
+          <t>output\screenshots\6_Galeries_Lafayette_Stage_Business_Analyst_F_H.png</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -787,353 +796,9 @@
       <c r="J7" s="3" t="inlineStr"/>
       <c r="K7" s="3" t="inlineStr"/>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Business Analyst (H/F)</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Davidson consulting</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>1 hour ago</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/business-analyst-h-f-at-davidson-consulting-4342654913</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>SQL, Jira, Confluence, Agile, Scrum, Gestion des parties prenantes, Recueil des besoins</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>output\screenshots\7_Davidson_consulting_Business_Analyst_(H_F).png</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Business Analyst Salesforce (H/F)</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>YEVO</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>23 hours ago</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/business-analyst-salesforce-h-f-at-yevo-4456807402</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Excel, Jira, Tableau, UML, Salesforce, Confluence, Agile, Scrum, Gestion des parties prenantes, Recueil des besoins, Gestion de projet, Compétences en communication</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>output\screenshots\8_YEVO_Business_Analyst_Salesforce_(H_F).png</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Business analyst</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Bending Spoons</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>19 hours ago</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/business-analyst-at-bending-spoons-4456804682</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Excel, Anglais</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>output\screenshots\9_Bending_Spoons_Business_analyst.png</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Data Analyst</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>papernest</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>5 hours ago</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/data-analyst-at-papernest-4458178575</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>SQL, Tableau, Français, Anglais</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>output\screenshots\10_papernest_Data_Analyst.png</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>Business Analyst - Base de données</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>act digital EMEA - Alter Solutions</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>9 hours ago</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/business-analyst-base-de-donn%C3%A9es-at-act-digital-emea-alter-solutions-4455826741</t>
-        </is>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>SQL, MS Visio, Agile, Gestion des parties prenantes, Recueil des besoins</t>
-        </is>
-      </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>output\screenshots\11_act_digital_EMEA_-_Alter_Solutions_Business_Analyst_-_Base_de_données.png</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Business Analyst Fonctionnel - Toulouse- F/H</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Free-Work</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>4 hours ago</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/business-analyst-fonctionnel-toulouse-f-h-at-free-work-4455849523</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>Excel, SAP, Agile, Scrum, Gestion des parties prenantes, Recueil des besoins, Gestion de projet</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>output\screenshots\12_Free-Work_Business_Analyst_Fonctionnel_-_Toulouse-_F_H.png</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Business Analyst / Consultant E-Commerce (H/F)</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>SQLI</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>21 hours ago</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/business-analyst-consultant-e-commerce-h-f-at-sqli-4390330065</t>
-        </is>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>SQL, Recueil des besoins, Compétences en communication</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>output\screenshots\13_SQLI_Business_Analyst_Consultant_E-Commerce_(H_F).png</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>Business Analyste technique – Assurance non vie (F/H)</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>BPCE Solutions informatiques</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>4 hours ago</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>https://fr.linkedin.com/jobs/view/business-analyste-technique-%E2%80%93-assurance-non-vie-f-h-at-bpce-solutions-informatiques-4428504183</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Jira, Confluence, MS Visio, Agile, DevOps, Recueil des besoins, Compétences en communication, Français, Anglais</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>output\screenshots\14_BPCE_Solutions_informatiques_Business_Analyste_technique_–_Assurance_non_vie_(F_H).png</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>À postuler</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Erreur" error="Saisie non valide" promptTitle="Statut Candidature" prompt="Veuillez choisir un statut dans la liste" type="list">
+    <dataValidation sqref="H2:H7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Erreur" error="Saisie non valide" promptTitle="Statut Candidature" prompt="Veuillez choisir un statut dans la liste" type="list">
       <formula1>"À postuler,Postulé,Entretien,Refusé,Offre reçue"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1150,22 +815,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1177,7 +826,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1222,20 +871,20 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Recueil des besoins</t>
+          <t>Anglais</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Compétence Professionnelle / Soft Skill</t>
+          <t>Langue</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>71.4%</t>
+          <t>83.3%</t>
         </is>
       </c>
     </row>
@@ -1247,7 +896,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>Power BI</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1256,11 +905,11 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>57.1%</t>
+          <t>66.7%</t>
         </is>
       </c>
     </row>
@@ -1272,7 +921,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>SQL</t>
+          <t>MS Visio</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -1281,11 +930,11 @@
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>35.7%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -1297,20 +946,20 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Gestion des parties prenantes</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Compétence Professionnelle / Soft Skill</t>
+          <t>Outil Technique / Logiciel</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>35.7%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -1322,7 +971,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Compétences en communication</t>
+          <t>Analyse de données</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1331,11 +980,11 @@
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>35.7%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -1347,20 +996,20 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Agile</t>
+          <t>Tableau</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Méthodologie / Framework</t>
+          <t>Outil Technique / Logiciel</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>35.7%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -1372,20 +1021,20 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Tableau</t>
+          <t>Gestion de projet</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Outil Technique / Logiciel</t>
+          <t>Compétence Professionnelle / Soft Skill</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>28.6%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -1397,20 +1046,20 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Anglais</t>
+          <t>Gestion du changement</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Langue</t>
+          <t>Compétence Professionnelle / Soft Skill</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>28.6%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1071,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>MS Visio</t>
+          <t>SQL</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1431,11 +1080,11 @@
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1447,20 +1096,20 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Confluence</t>
+          <t>Français</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Outil Technique / Logiciel</t>
+          <t>Langue</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1121,7 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Jira</t>
+          <t>PowerPoint</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1481,11 +1130,11 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1497,20 +1146,20 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Scrum</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Méthodologie / Framework</t>
+          <t>Outil Technique / Logiciel</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1171,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Gestion de projet</t>
+          <t>Gestion des parties prenantes</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1531,11 +1180,11 @@
         </is>
       </c>
       <c r="D14" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>21.4%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1547,20 +1196,20 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Français</t>
+          <t>Recueil des besoins</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Langue</t>
+          <t>Compétence Professionnelle / Soft Skill</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1572,7 +1221,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Python</t>
+          <t>SharePoint</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1581,11 +1230,11 @@
         </is>
       </c>
       <c r="D16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>
@@ -1597,145 +1246,20 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Power BI</t>
+          <t>Compétences en communication</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Outil Technique / Logiciel</t>
+          <t>Compétence Professionnelle / Soft Skill</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>14.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Top 17</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Salesforce</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Outil Technique / Logiciel</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>14.3%</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Top 18</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>R</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Outil Technique / Logiciel</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>7.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Top 19</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>UML</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Outil Technique / Logiciel</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>7.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Top 20</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>SAP</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Outil Technique / Logiciel</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>7.1%</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Top 21</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>DevOps</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Méthodologie / Framework</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>7.1%</t>
+          <t>16.7%</t>
         </is>
       </c>
     </row>

</xml_diff>